<commit_message>
Separated eval and train code
</commit_message>
<xml_diff>
--- a/outputs/CNN_output.xlsx
+++ b/outputs/CNN_output.xlsx
@@ -964,7 +964,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>sigatoka</t>
+          <t>pestalotiopsis</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1312,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>pestalotiopsis</t>
+          <t>cordona</t>
         </is>
       </c>
     </row>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>cordona</t>
+          <t>pestalotiopsis</t>
         </is>
       </c>
     </row>

</xml_diff>